<commit_message>
Update marginal summary references to Table 6
</commit_message>
<xml_diff>
--- a/Root/reproducibility/patient_mil_v1/model_selection/Supplementary_Table_S1.xlsx
+++ b/Root/reproducibility/patient_mil_v1/model_selection/Supplementary_Table_S1.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S1 All Candidates" sheetId="1" r:id="Rcf7c4c2c7dff4b41"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Selected Check" sheetId="2" r:id="Rc7c8271c8f5c4830"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Marginal Check" sheetId="3" r:id="R27fb4fb5b3f74729"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="4" r:id="R5a094a12d0f44f02"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S1 All Candidates" sheetId="1" r:id="Rc9a3f265205e4b9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Selected Check" sheetId="2" r:id="Rd05e029113244e65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Marginal Check" sheetId="3" r:id="R474442c8d3f6473a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="4" r:id="Rdead27b20cd64cb1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -34427,7 +34427,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea301eb378294237"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ba254cc6d20411b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -34611,7 +34611,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce374dbc6d8249d4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R069d5f4c4b4142de"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -34664,16 +34664,16 @@
         <x:v>Accuracy sample SD</x:v>
       </x:c>
       <x:c r="J1" s="44" t="str">
-        <x:v>Table 5 AUROC</x:v>
+        <x:v>Table 6 AUROC</x:v>
       </x:c>
       <x:c r="K1" s="44" t="str">
-        <x:v>Table 5 AUPRC</x:v>
+        <x:v>Table 6 AUPRC</x:v>
       </x:c>
       <x:c r="L1" s="44" t="str">
-        <x:v>Table 5 accuracy</x:v>
+        <x:v>Table 6 accuracy</x:v>
       </x:c>
       <x:c r="M1" s="44" t="str">
-        <x:v>Matches Table 5</x:v>
+        <x:v>Matches Table 6</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -35253,7 +35253,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re553ec6a518e4af8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R90b170fc84d8468d"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>